<commit_message>
Commit N6 insert news end devices in the network
</commit_message>
<xml_diff>
--- a/3_N4_Armazenamento/Parametros/Pacote_DL_UL.xlsx
+++ b/3_N4_Armazenamento/Parametros/Pacote_DL_UL.xlsx
@@ -446,7 +446,7 @@
         <v>0</v>
       </c>
       <c r="C2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D2" t="s">
         <v>11</v>
@@ -472,7 +472,7 @@
         <v>1</v>
       </c>
       <c r="C3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" t="s">
         <v>12</v>
@@ -498,7 +498,7 @@
         <v>2</v>
       </c>
       <c r="C4">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
@@ -524,7 +524,7 @@
         <v>3</v>
       </c>
       <c r="C5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D5" t="s">
         <v>14</v>
@@ -550,7 +550,7 @@
         <v>4</v>
       </c>
       <c r="C6">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
         <v>17</v>
@@ -573,7 +573,7 @@
         <v>5</v>
       </c>
       <c r="C7">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
         <v>18</v>
@@ -596,7 +596,7 @@
         <v>6</v>
       </c>
       <c r="C8">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D8" t="s">
         <v>16</v>
@@ -619,7 +619,7 @@
         <v>7</v>
       </c>
       <c r="C9">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D9" t="s">
         <v>15</v>
@@ -642,7 +642,7 @@
         <v>8</v>
       </c>
       <c r="C10">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D10" t="s">
         <v>19</v>
@@ -668,7 +668,7 @@
         <v>9</v>
       </c>
       <c r="C11">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D11" t="s">
         <v>20</v>
@@ -691,7 +691,7 @@
         <v>10</v>
       </c>
       <c r="C12">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -717,7 +717,7 @@
         <v>11</v>
       </c>
       <c r="C13">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F13" t="s">
         <v>0</v>
@@ -737,7 +737,7 @@
         <v>12</v>
       </c>
       <c r="C14">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F14" t="s">
         <v>0</v>
@@ -757,7 +757,7 @@
         <v>13</v>
       </c>
       <c r="C15">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="F15" t="s">
         <v>0</v>
@@ -777,7 +777,7 @@
         <v>14</v>
       </c>
       <c r="C16">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F16" t="s">
         <v>0</v>
@@ -797,7 +797,7 @@
         <v>15</v>
       </c>
       <c r="C17">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F17" t="s">
         <v>0</v>
@@ -817,7 +817,7 @@
         <v>16</v>
       </c>
       <c r="C18">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
         <v>0</v>
@@ -837,7 +837,7 @@
         <v>17</v>
       </c>
       <c r="C19">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F19" t="s">
         <v>0</v>
@@ -857,7 +857,7 @@
         <v>18</v>
       </c>
       <c r="C20">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F20" t="s">
         <v>0</v>
@@ -877,7 +877,7 @@
         <v>19</v>
       </c>
       <c r="C21">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F21" t="s">
         <v>0</v>
@@ -897,7 +897,7 @@
         <v>20</v>
       </c>
       <c r="C22">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F22" t="s">
         <v>0</v>
@@ -917,7 +917,7 @@
         <v>21</v>
       </c>
       <c r="C23">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F23" t="s">
         <v>0</v>
@@ -937,7 +937,7 @@
         <v>22</v>
       </c>
       <c r="C24">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F24" t="s">
         <v>0</v>
@@ -957,7 +957,7 @@
         <v>23</v>
       </c>
       <c r="C25">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F25" t="s">
         <v>0</v>
@@ -977,7 +977,7 @@
         <v>24</v>
       </c>
       <c r="C26">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F26" t="s">
         <v>0</v>
@@ -997,7 +997,7 @@
         <v>25</v>
       </c>
       <c r="C27">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F27" t="s">
         <v>0</v>
@@ -1017,7 +1017,7 @@
         <v>26</v>
       </c>
       <c r="C28">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F28" t="s">
         <v>0</v>
@@ -1037,7 +1037,7 @@
         <v>27</v>
       </c>
       <c r="C29">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="F29" t="s">
         <v>0</v>
@@ -1057,7 +1057,7 @@
         <v>28</v>
       </c>
       <c r="C30">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F30" t="s">
         <v>0</v>
@@ -1077,7 +1077,7 @@
         <v>29</v>
       </c>
       <c r="C31">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F31" t="s">
         <v>0</v>

</xml_diff>